<commit_message>
update for May 2026
</commit_message>
<xml_diff>
--- a/NBDHE Subject Breakdown.xlsx
+++ b/NBDHE Subject Breakdown.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\18005262\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE1C221-9A7C-40AA-894D-738948CF677D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937BEC4F-BAF6-4D39-9C65-DEF081978932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="1440" windowWidth="19950" windowHeight="13305" activeTab="1" xr2:uid="{E733ED90-E2C8-4DFA-A854-71184709D5C0}"/>
+    <workbookView xWindow="33150" yWindow="1605" windowWidth="19950" windowHeight="13305" activeTab="1" xr2:uid="{E733ED90-E2C8-4DFA-A854-71184709D5C0}"/>
   </bookViews>
   <sheets>
     <sheet name="How to Use" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
     <author>Wendy D Heimann</author>
   </authors>
   <commentList>
-    <comment ref="AT1" authorId="0" shapeId="0" xr:uid="{8E362791-52EB-4E9B-882D-F6A80812C50C}">
+    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{8E362791-52EB-4E9B-882D-F6A80812C50C}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{9CAB04E5-A305-48C0-9D91-DDBA6B2E3634}">
+    <comment ref="I18" authorId="0" shapeId="0" xr:uid="{9CAB04E5-A305-48C0-9D91-DDBA6B2E3634}">
       <text>
         <r>
           <rPr>
@@ -93,7 +93,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA18" authorId="0" shapeId="0" xr:uid="{5AB4E218-AC89-4ACA-9590-C14D343CD161}">
+    <comment ref="AB18" authorId="0" shapeId="0" xr:uid="{5AB4E218-AC89-4ACA-9590-C14D343CD161}">
       <text>
         <r>
           <rPr>
@@ -118,7 +118,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH18" authorId="0" shapeId="0" xr:uid="{6C7A0DB6-473C-40E9-88DF-CFC02AF305D1}">
+    <comment ref="AI18" authorId="0" shapeId="0" xr:uid="{6C7A0DB6-473C-40E9-88DF-CFC02AF305D1}">
       <text>
         <r>
           <rPr>
@@ -143,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL18" authorId="0" shapeId="0" xr:uid="{FF80E043-AB05-42EF-B310-15578A867E69}">
+    <comment ref="AM18" authorId="0" shapeId="0" xr:uid="{FF80E043-AB05-42EF-B310-15578A867E69}">
       <text>
         <r>
           <rPr>
@@ -168,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AM18" authorId="0" shapeId="0" xr:uid="{2D056A91-DFC9-4F19-8839-996FF1451DB1}">
+    <comment ref="AN18" authorId="0" shapeId="0" xr:uid="{2D056A91-DFC9-4F19-8839-996FF1451DB1}">
       <text>
         <r>
           <rPr>
@@ -194,7 +194,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN18" authorId="0" shapeId="0" xr:uid="{3F6E2DFC-6D8A-41A6-854E-5A4F59A11920}">
+    <comment ref="AO18" authorId="0" shapeId="0" xr:uid="{3F6E2DFC-6D8A-41A6-854E-5A4F59A11920}">
       <text>
         <r>
           <rPr>
@@ -220,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AO18" authorId="0" shapeId="0" xr:uid="{8FD5A144-EBB0-48E5-9646-2EE38A1BD71C}">
+    <comment ref="AP18" authorId="0" shapeId="0" xr:uid="{8FD5A144-EBB0-48E5-9646-2EE38A1BD71C}">
       <text>
         <r>
           <rPr>
@@ -246,7 +246,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AS18" authorId="0" shapeId="0" xr:uid="{EA492413-C88C-49BE-A24D-EB97639284D4}">
+    <comment ref="AT18" authorId="0" shapeId="0" xr:uid="{EA492413-C88C-49BE-A24D-EB97639284D4}">
       <text>
         <r>
           <rPr>
@@ -272,7 +272,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AU18" authorId="0" shapeId="0" xr:uid="{1A7309AD-2F00-4559-9560-833E20CF1785}">
+    <comment ref="AV18" authorId="0" shapeId="0" xr:uid="{1A7309AD-2F00-4559-9560-833E20CF1785}">
       <text>
         <r>
           <rPr>
@@ -298,7 +298,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AX18" authorId="0" shapeId="0" xr:uid="{DC907309-8913-4275-904F-A04B499FA001}">
+    <comment ref="AY18" authorId="0" shapeId="0" xr:uid="{DC907309-8913-4275-904F-A04B499FA001}">
       <text>
         <r>
           <rPr>
@@ -323,7 +323,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG18" authorId="0" shapeId="0" xr:uid="{CBA21150-414F-4FAB-AAF2-8C8F542659CC}">
+    <comment ref="BH18" authorId="0" shapeId="0" xr:uid="{CBA21150-414F-4FAB-AAF2-8C8F542659CC}">
       <text>
         <r>
           <rPr>
@@ -349,7 +349,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ18" authorId="0" shapeId="0" xr:uid="{0260BC2A-568D-4D13-9CCF-D49ED7F09A6F}">
+    <comment ref="BK18" authorId="0" shapeId="0" xr:uid="{0260BC2A-568D-4D13-9CCF-D49ED7F09A6F}">
       <text>
         <r>
           <rPr>
@@ -375,7 +375,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK18" authorId="0" shapeId="0" xr:uid="{2E418255-44B2-4493-BCF6-B130A2D95813}">
+    <comment ref="BL18" authorId="0" shapeId="0" xr:uid="{2E418255-44B2-4493-BCF6-B130A2D95813}">
       <text>
         <r>
           <rPr>
@@ -405,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
   <si>
     <t>Anatomic Science</t>
   </si>
@@ -720,6 +720,9 @@
   </si>
   <si>
     <t>Pharmacology*</t>
+  </si>
+  <si>
+    <t>6/25-5/26</t>
   </si>
 </sst>
 </file>
@@ -807,7 +810,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -831,7 +834,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1189,387 +1191,390 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{723F4256-9B45-4CD1-A91B-7679EC611E87}">
-  <dimension ref="A1:BZ21"/>
+  <dimension ref="A1:CA21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="17" width="12.7109375" style="2" customWidth="1"/>
-    <col min="18" max="80" width="12.7109375" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="18" width="12.7109375" style="2" customWidth="1"/>
+    <col min="19" max="81" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AC1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AE1" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AF1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AG1" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AH1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AI1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AJ1" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="AK1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AM1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="AM1" s="6" t="s">
+      <c r="AN1" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AO1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="AO1" s="6" t="s">
+      <c r="AP1" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AP1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="AQ1" s="6" t="s">
+      <c r="AR1" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="AR1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="AS1" s="6" t="s">
+      <c r="AT1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="AT1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="AU1" s="6" t="s">
+      <c r="AV1" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="AV1" s="6" t="s">
+      <c r="AW1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="AW1" s="6" t="s">
+      <c r="AX1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="AX1" s="6" t="s">
+      <c r="AY1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="AY1" s="6" t="s">
+      <c r="AZ1" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="AZ1" s="6" t="s">
+      <c r="BA1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="BA1" s="6" t="s">
+      <c r="BB1" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="BB1" s="6" t="s">
+      <c r="BC1" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="BC1" s="6" t="s">
+      <c r="BD1" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="BD1" s="6" t="s">
+      <c r="BE1" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="BE1" s="6" t="s">
+      <c r="BF1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="BF1" s="6" t="s">
+      <c r="BG1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="BG1" s="6" t="s">
+      <c r="BH1" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="BH1" s="6" t="s">
+      <c r="BI1" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="BI1" s="6" t="s">
+      <c r="BJ1" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="BJ1" s="6" t="s">
+      <c r="BK1" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="BK1" s="6" t="s">
+      <c r="BL1" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="BL1" s="6" t="s">
+      <c r="BM1" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="BM1" s="6" t="s">
+      <c r="BN1" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="BN1" s="6" t="s">
+      <c r="BO1" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="BO1" s="6" t="s">
+      <c r="BP1" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="BP1" s="6" t="s">
+      <c r="BQ1" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="BQ1" s="6" t="s">
+      <c r="BR1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="BR1" s="6" t="s">
+      <c r="BS1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="BS1" s="6" t="s">
+      <c r="BT1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="BT1" s="6" t="s">
+      <c r="BU1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="BU1" s="6" t="s">
+      <c r="BV1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="BV1" s="6" t="s">
+      <c r="BW1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="BW1" s="6" t="s">
+      <c r="BX1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="BX1" s="6" t="s">
+      <c r="BY1" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="BY1" s="6" t="s">
+      <c r="BZ1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
     </row>
-    <row r="2" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
+        <v>-0.18</v>
+      </c>
+      <c r="C2">
         <v>-0.23</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>-0.85</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>-0.77</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>-0.79</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>-0.78</v>
-      </c>
-      <c r="G2" s="2">
-        <v>-0.74</v>
       </c>
       <c r="H2" s="2">
         <v>-0.74</v>
       </c>
       <c r="I2" s="2">
+        <v>-0.74</v>
+      </c>
+      <c r="J2" s="2">
         <v>-1.78</v>
       </c>
-      <c r="J2" s="2">
+      <c r="K2" s="2">
         <v>-1.59</v>
       </c>
-      <c r="K2" s="2">
+      <c r="L2" s="2">
         <v>-1.56</v>
       </c>
-      <c r="L2" s="2">
+      <c r="M2" s="2">
         <v>-1.69</v>
       </c>
-      <c r="M2" s="2">
+      <c r="N2" s="2">
         <v>-1.6</v>
       </c>
-      <c r="N2" s="2">
+      <c r="O2" s="2">
         <v>-1.82</v>
       </c>
-      <c r="O2" s="2">
+      <c r="P2" s="2">
         <v>-1.1299999999999999</v>
-      </c>
-      <c r="P2" s="2">
-        <v>-1.1000000000000001</v>
       </c>
       <c r="Q2" s="2">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="2">
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="S2">
         <v>-1.0900000000000001</v>
-      </c>
-      <c r="S2">
-        <v>-1.1599999999999999</v>
       </c>
       <c r="T2">
         <v>-1.1599999999999999</v>
       </c>
       <c r="U2">
+        <v>-1.1599999999999999</v>
+      </c>
+      <c r="V2">
         <v>-1.19</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>-1.69</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>-1.66</v>
       </c>
-      <c r="X2">
+      <c r="Y2">
         <v>-1.01</v>
       </c>
-      <c r="Y2">
+      <c r="Z2">
         <v>-1.02</v>
       </c>
-      <c r="Z2">
+      <c r="AA2">
         <v>-0.81</v>
       </c>
-      <c r="AA2">
+      <c r="AB2">
         <v>-0.9</v>
       </c>
-      <c r="AB2">
+      <c r="AC2">
         <v>-0.59</v>
       </c>
-      <c r="AC2">
+      <c r="AD2">
         <v>-0.46</v>
       </c>
-      <c r="AD2">
+      <c r="AE2">
         <v>-0.45</v>
       </c>
-      <c r="AE2">
+      <c r="AF2">
         <v>-0.47</v>
       </c>
-      <c r="AF2">
+      <c r="AG2">
         <v>-0.45</v>
       </c>
-      <c r="AG2">
+      <c r="AH2">
         <v>-0.36</v>
       </c>
-      <c r="AH2">
+      <c r="AI2">
         <v>-0.06</v>
       </c>
-      <c r="AI2">
+      <c r="AJ2">
         <v>-0.81</v>
       </c>
-      <c r="AJ2">
+      <c r="AK2">
         <v>-1.75</v>
       </c>
-      <c r="AK2">
+      <c r="AL2">
         <v>-1.76</v>
       </c>
-      <c r="AL2">
+      <c r="AM2">
         <v>-1.84</v>
       </c>
-      <c r="AM2">
+      <c r="AN2">
         <v>-1.82</v>
       </c>
-      <c r="AN2">
+      <c r="AO2">
         <v>-1.81</v>
       </c>
-      <c r="AO2">
+      <c r="AP2">
         <v>-1.92</v>
       </c>
-      <c r="AP2">
+      <c r="AQ2">
         <v>-1.83</v>
       </c>
-      <c r="AQ2">
+      <c r="AR2">
         <v>-1.82</v>
-      </c>
-      <c r="AR2">
-        <v>-1.79</v>
       </c>
       <c r="AS2">
         <v>-1.79</v>
       </c>
       <c r="AT2">
-        <v>0</v>
+        <v>-1.79</v>
       </c>
       <c r="AU2">
         <v>0</v>
@@ -1647,36 +1652,39 @@
         <v>0</v>
       </c>
       <c r="BT2">
+        <v>0</v>
+      </c>
+      <c r="BU2">
         <v>-0.42</v>
       </c>
-      <c r="BU2">
+      <c r="BV2">
         <v>-0.6</v>
       </c>
-      <c r="BV2">
+      <c r="BW2">
         <v>-0.43</v>
       </c>
-      <c r="BW2">
+      <c r="BX2">
         <v>-0.51</v>
       </c>
-      <c r="BX2">
+      <c r="BY2">
         <v>-0.71</v>
       </c>
-      <c r="BY2">
+      <c r="BZ2">
         <v>-0.86</v>
       </c>
     </row>
-    <row r="3" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:79" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3">
+        <v>1.25</v>
+      </c>
+      <c r="C3">
         <v>1.03</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>0.59</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0.66</v>
       </c>
       <c r="E3" s="2">
         <v>0.66</v>
@@ -1685,125 +1693,125 @@
         <v>0.66</v>
       </c>
       <c r="G3" s="2">
+        <v>0.66</v>
+      </c>
+      <c r="H3" s="2">
         <v>0.81</v>
       </c>
-      <c r="H3" s="2">
+      <c r="I3" s="2">
         <v>0.66</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>-0.34</v>
       </c>
-      <c r="J3" s="2">
+      <c r="K3" s="2">
         <v>-0.33</v>
       </c>
-      <c r="K3" s="2">
+      <c r="L3" s="2">
         <v>-0.32</v>
-      </c>
-      <c r="L3" s="2">
-        <v>-0.53</v>
       </c>
       <c r="M3" s="2">
         <v>-0.53</v>
       </c>
       <c r="N3" s="2">
+        <v>-0.53</v>
+      </c>
+      <c r="O3" s="2">
         <v>-0.72</v>
       </c>
-      <c r="O3" s="2">
+      <c r="P3" s="2">
         <v>-0.39</v>
-      </c>
-      <c r="P3" s="2">
-        <v>-0.25</v>
       </c>
       <c r="Q3" s="2">
         <v>-0.25</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="2">
         <v>-0.25</v>
       </c>
       <c r="S3">
+        <v>-0.25</v>
+      </c>
+      <c r="T3">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>-0.56999999999999995</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>-0.7</v>
       </c>
-      <c r="V3">
+      <c r="W3">
         <v>-1.07</v>
       </c>
-      <c r="W3">
+      <c r="X3">
         <v>-0.92</v>
       </c>
-      <c r="X3">
+      <c r="Y3">
         <v>-0.98</v>
       </c>
-      <c r="Y3">
+      <c r="Z3">
         <v>-0.96</v>
       </c>
-      <c r="Z3">
+      <c r="AA3">
         <v>-0.9</v>
       </c>
-      <c r="AA3">
+      <c r="AB3">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>-0.45</v>
       </c>
-      <c r="AC3">
+      <c r="AD3">
         <v>-0.15</v>
-      </c>
-      <c r="AD3">
-        <v>-0.16</v>
       </c>
       <c r="AE3">
         <v>-0.16</v>
       </c>
       <c r="AF3">
+        <v>-0.16</v>
+      </c>
+      <c r="AG3">
         <v>-0.15</v>
       </c>
-      <c r="AG3">
+      <c r="AH3">
         <v>-0.02</v>
       </c>
-      <c r="AH3">
+      <c r="AI3">
         <v>0.09</v>
       </c>
-      <c r="AI3">
+      <c r="AJ3">
         <v>-0.64</v>
       </c>
-      <c r="AJ3">
+      <c r="AK3">
         <v>-0.94</v>
       </c>
-      <c r="AK3">
+      <c r="AL3">
         <v>-0.91</v>
       </c>
-      <c r="AL3">
+      <c r="AM3">
         <v>-0.85</v>
       </c>
-      <c r="AM3">
+      <c r="AN3">
         <v>-1.22</v>
       </c>
-      <c r="AN3">
+      <c r="AO3">
         <v>-1.54</v>
       </c>
-      <c r="AO3">
+      <c r="AP3">
         <v>-2.16</v>
       </c>
-      <c r="AP3">
+      <c r="AQ3">
         <v>-1.98</v>
       </c>
-      <c r="AQ3">
+      <c r="AR3">
         <v>-2</v>
       </c>
-      <c r="AR3">
+      <c r="AS3">
         <v>-1.96</v>
       </c>
-      <c r="AS3">
+      <c r="AT3">
         <v>-1.94</v>
       </c>
-      <c r="AT3">
-        <v>0</v>
-      </c>
       <c r="AU3">
         <v>0</v>
       </c>
@@ -1880,163 +1888,166 @@
         <v>0</v>
       </c>
       <c r="BT3">
+        <v>0</v>
+      </c>
+      <c r="BU3">
         <v>-0.59</v>
       </c>
-      <c r="BU3">
+      <c r="BV3">
         <v>-0.47</v>
       </c>
-      <c r="BV3">
+      <c r="BW3">
         <v>-0.24</v>
       </c>
-      <c r="BW3">
+      <c r="BX3">
         <v>-0.35</v>
       </c>
-      <c r="BX3">
+      <c r="BY3">
         <v>-0.38</v>
       </c>
-      <c r="BY3">
+      <c r="BZ3">
         <v>-0.46</v>
       </c>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:79" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
+        <v>0.96</v>
+      </c>
+      <c r="C4">
         <v>1.01</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>0.97</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4" s="2">
         <v>1.03</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1.02</v>
       </c>
       <c r="F4" s="2">
         <v>1.02</v>
       </c>
       <c r="G4" s="2">
+        <v>1.02</v>
+      </c>
+      <c r="H4" s="2">
         <v>0.65</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>0.83</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>-0.41</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>0.11</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>0.12</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="2">
         <v>-0.13</v>
       </c>
-      <c r="M4" s="2">
+      <c r="N4" s="2">
         <v>-0.15</v>
       </c>
-      <c r="N4" s="2">
+      <c r="O4" s="2">
         <v>-0.53</v>
       </c>
-      <c r="O4" s="2">
+      <c r="P4" s="2">
         <v>-0.78</v>
       </c>
-      <c r="P4" s="2">
+      <c r="Q4" s="2">
         <v>-0.35</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="R4" s="2">
         <v>-0.36</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>-0.35</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>-0.05</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>-0.04</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>-0.05</v>
       </c>
-      <c r="V4">
+      <c r="W4">
         <v>-0.45</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <v>-0.28000000000000003</v>
       </c>
-      <c r="X4">
+      <c r="Y4">
         <v>0.56000000000000005</v>
       </c>
-      <c r="Y4">
+      <c r="Z4">
         <v>0.6</v>
       </c>
-      <c r="Z4">
+      <c r="AA4">
         <v>0.93</v>
       </c>
-      <c r="AA4">
+      <c r="AB4">
         <v>1.08</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
         <v>0.57999999999999996</v>
-      </c>
-      <c r="AC4">
-        <v>0.84</v>
       </c>
       <c r="AD4">
         <v>0.84</v>
       </c>
       <c r="AE4">
+        <v>0.84</v>
+      </c>
+      <c r="AF4">
         <v>0.85</v>
       </c>
-      <c r="AF4">
+      <c r="AG4">
         <v>0.86</v>
       </c>
-      <c r="AG4">
+      <c r="AH4">
         <v>1</v>
       </c>
-      <c r="AH4">
+      <c r="AI4">
         <v>0.95</v>
       </c>
-      <c r="AI4">
+      <c r="AJ4">
         <v>0.13</v>
       </c>
-      <c r="AJ4">
+      <c r="AK4">
         <v>-1.18</v>
       </c>
-      <c r="AK4">
+      <c r="AL4">
         <v>-1.17</v>
       </c>
-      <c r="AL4">
+      <c r="AM4">
         <v>-1.36</v>
       </c>
-      <c r="AM4">
+      <c r="AN4">
         <v>-1.44</v>
       </c>
-      <c r="AN4">
+      <c r="AO4">
         <v>-1.43</v>
       </c>
-      <c r="AO4">
+      <c r="AP4">
         <v>-1.85</v>
-      </c>
-      <c r="AP4">
-        <v>-2.06</v>
       </c>
       <c r="AQ4">
         <v>-2.06</v>
       </c>
       <c r="AR4">
+        <v>-2.06</v>
+      </c>
+      <c r="AS4">
         <v>-2.04</v>
       </c>
-      <c r="AS4">
+      <c r="AT4">
         <v>-2.0099999999999998</v>
       </c>
-      <c r="AT4">
-        <v>0</v>
-      </c>
       <c r="AU4">
         <v>0</v>
       </c>
@@ -2113,36 +2124,39 @@
         <v>0</v>
       </c>
       <c r="BT4">
+        <v>0</v>
+      </c>
+      <c r="BU4">
         <v>-0.43</v>
       </c>
-      <c r="BU4">
+      <c r="BV4">
         <v>-0.2</v>
       </c>
-      <c r="BV4">
+      <c r="BW4">
         <v>-0.11</v>
       </c>
-      <c r="BW4">
+      <c r="BX4">
         <v>-0.35</v>
       </c>
-      <c r="BX4">
+      <c r="BY4">
         <v>-0.36</v>
       </c>
-      <c r="BY4">
+      <c r="BZ4">
         <v>-0.17</v>
       </c>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
+        <v>0.61</v>
+      </c>
+      <c r="C5">
         <v>0.56000000000000005</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>-0.04</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.15</v>
       </c>
       <c r="E5" s="2">
         <v>0.15</v>
@@ -2151,73 +2165,73 @@
         <v>0.15</v>
       </c>
       <c r="G5" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H5" s="2">
         <v>-0.05</v>
       </c>
-      <c r="H5" s="2">
+      <c r="I5" s="2">
         <v>0.04</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <v>-1.38</v>
       </c>
-      <c r="J5" s="2">
+      <c r="K5" s="2">
         <v>-1.32</v>
       </c>
-      <c r="K5" s="2">
+      <c r="L5" s="2">
         <v>-1.29</v>
       </c>
-      <c r="L5" s="2">
+      <c r="M5" s="2">
         <v>-1.36</v>
       </c>
-      <c r="M5" s="2">
+      <c r="N5" s="2">
         <v>-1.32</v>
       </c>
-      <c r="N5" s="2">
+      <c r="O5" s="2">
         <v>-1.55</v>
       </c>
-      <c r="O5" s="2">
+      <c r="P5" s="2">
         <v>-1.71</v>
       </c>
-      <c r="P5" s="2">
+      <c r="Q5" s="2">
         <v>-1.67</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="R5" s="2">
         <v>-1.68</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>-1.67</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>-1.6</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>-1.58</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <v>-1.65</v>
       </c>
-      <c r="V5">
+      <c r="W5">
         <v>-2.21</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <v>-2.2799999999999998</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <v>-1.6</v>
       </c>
-      <c r="Y5">
+      <c r="Z5">
         <v>-1.65</v>
       </c>
-      <c r="Z5">
+      <c r="AA5">
         <v>-1.78</v>
       </c>
-      <c r="AA5">
+      <c r="AB5">
         <v>-1.35</v>
       </c>
-      <c r="AB5">
+      <c r="AC5">
         <v>-1.2</v>
-      </c>
-      <c r="AC5">
-        <v>-0.92</v>
       </c>
       <c r="AD5">
         <v>-0.92</v>
@@ -2229,47 +2243,47 @@
         <v>-0.92</v>
       </c>
       <c r="AG5">
+        <v>-0.92</v>
+      </c>
+      <c r="AH5">
         <v>-0.85</v>
       </c>
-      <c r="AH5">
+      <c r="AI5">
         <v>-0.67</v>
       </c>
-      <c r="AI5">
+      <c r="AJ5">
         <v>-1.19</v>
       </c>
-      <c r="AJ5">
+      <c r="AK5">
         <v>-1.9</v>
       </c>
-      <c r="AK5">
+      <c r="AL5">
         <v>-1.87</v>
       </c>
-      <c r="AL5">
+      <c r="AM5">
         <v>-1.73</v>
       </c>
-      <c r="AM5">
+      <c r="AN5">
         <v>-2.0499999999999998</v>
       </c>
-      <c r="AN5">
+      <c r="AO5">
         <v>-2.15</v>
       </c>
-      <c r="AO5">
+      <c r="AP5">
         <v>-2.4300000000000002</v>
       </c>
-      <c r="AP5">
+      <c r="AQ5">
         <v>-2.2799999999999998</v>
       </c>
-      <c r="AQ5">
+      <c r="AR5">
         <v>-2.2599999999999998</v>
       </c>
-      <c r="AR5">
+      <c r="AS5">
         <v>-2.1800000000000002</v>
       </c>
-      <c r="AS5">
+      <c r="AT5">
         <v>-2.19</v>
       </c>
-      <c r="AT5">
-        <v>0</v>
-      </c>
       <c r="AU5">
         <v>0</v>
       </c>
@@ -2346,163 +2360,166 @@
         <v>0</v>
       </c>
       <c r="BT5">
+        <v>0</v>
+      </c>
+      <c r="BU5">
         <v>-0.34</v>
       </c>
-      <c r="BU5">
+      <c r="BV5">
         <v>-0.38</v>
       </c>
-      <c r="BV5">
+      <c r="BW5">
         <v>-0.28999999999999998</v>
       </c>
-      <c r="BW5">
+      <c r="BX5">
         <v>-0.37</v>
       </c>
-      <c r="BX5">
+      <c r="BY5">
         <v>-0.74</v>
       </c>
-      <c r="BY5">
+      <c r="BZ5">
         <v>-0.81</v>
       </c>
     </row>
-    <row r="6" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>104</v>
       </c>
       <c r="B6">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="C6">
         <v>1</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>0.45</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="2">
         <v>0.48</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0.47</v>
       </c>
       <c r="F6" s="2">
         <v>0.47</v>
       </c>
       <c r="G6" s="2">
+        <v>0.47</v>
+      </c>
+      <c r="H6" s="2">
         <v>0.23</v>
       </c>
-      <c r="H6" s="2">
+      <c r="I6" s="2">
         <v>0.26</v>
       </c>
-      <c r="I6" s="2">
+      <c r="J6" s="2">
         <v>-1.02</v>
       </c>
-      <c r="J6" s="2">
+      <c r="K6" s="2">
         <v>-1.39</v>
       </c>
-      <c r="K6" s="2">
+      <c r="L6" s="2">
         <v>-1.36</v>
       </c>
-      <c r="L6" s="2">
+      <c r="M6" s="2">
         <v>-1.55</v>
       </c>
-      <c r="M6" s="2">
+      <c r="N6" s="2">
         <v>-1.53</v>
       </c>
-      <c r="N6" s="2">
+      <c r="O6" s="2">
         <v>-1.68</v>
       </c>
-      <c r="O6" s="2">
+      <c r="P6" s="2">
         <v>-1.79</v>
-      </c>
-      <c r="P6" s="2">
-        <v>-1.4</v>
       </c>
       <c r="Q6" s="2">
         <v>-1.4</v>
       </c>
-      <c r="R6">
+      <c r="R6" s="2">
         <v>-1.4</v>
       </c>
       <c r="S6">
+        <v>-1.4</v>
+      </c>
+      <c r="T6">
         <v>-1.29</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>-1.28</v>
       </c>
-      <c r="U6">
+      <c r="V6">
         <v>-1.06</v>
       </c>
-      <c r="V6">
+      <c r="W6">
         <v>-0.91</v>
       </c>
-      <c r="W6">
+      <c r="X6">
         <v>-1.33</v>
       </c>
-      <c r="X6">
+      <c r="Y6">
         <v>-0.91</v>
       </c>
-      <c r="Y6">
+      <c r="Z6">
         <v>-0.88</v>
       </c>
-      <c r="Z6">
+      <c r="AA6">
         <v>-0.8</v>
       </c>
-      <c r="AA6">
+      <c r="AB6">
         <v>-0.49</v>
       </c>
-      <c r="AB6">
+      <c r="AC6">
         <v>-0.48</v>
       </c>
-      <c r="AC6">
+      <c r="AD6">
         <v>-0.52</v>
       </c>
-      <c r="AD6">
+      <c r="AE6">
         <v>-0.51</v>
-      </c>
-      <c r="AE6">
-        <v>-0.49</v>
       </c>
       <c r="AF6">
         <v>-0.49</v>
       </c>
       <c r="AG6">
+        <v>-0.49</v>
+      </c>
+      <c r="AH6">
         <v>-0.64</v>
       </c>
-      <c r="AH6">
+      <c r="AI6">
         <v>-0.45</v>
       </c>
-      <c r="AI6">
+      <c r="AJ6">
         <v>-0.47</v>
       </c>
-      <c r="AJ6">
+      <c r="AK6">
         <v>-1.35</v>
       </c>
-      <c r="AK6">
+      <c r="AL6">
         <v>-1.33</v>
       </c>
-      <c r="AL6">
+      <c r="AM6">
         <v>-1.38</v>
       </c>
-      <c r="AM6">
+      <c r="AN6">
         <v>-1.7</v>
       </c>
-      <c r="AN6">
+      <c r="AO6">
         <v>-1.99</v>
       </c>
-      <c r="AO6">
+      <c r="AP6">
         <v>-1.96</v>
       </c>
-      <c r="AP6">
+      <c r="AQ6">
         <v>-1.52</v>
       </c>
-      <c r="AQ6">
+      <c r="AR6">
         <v>-1.49</v>
       </c>
-      <c r="AR6">
+      <c r="AS6">
         <v>-1.44</v>
       </c>
-      <c r="AS6">
+      <c r="AT6">
         <v>-1.45</v>
       </c>
-      <c r="AT6">
-        <v>0</v>
-      </c>
       <c r="AU6">
         <v>0</v>
       </c>
@@ -2579,36 +2596,39 @@
         <v>0</v>
       </c>
       <c r="BT6">
+        <v>0</v>
+      </c>
+      <c r="BU6">
         <v>0.82</v>
       </c>
-      <c r="BU6">
+      <c r="BV6">
         <v>1.1499999999999999</v>
       </c>
-      <c r="BV6">
+      <c r="BW6">
         <v>1.29</v>
       </c>
-      <c r="BW6">
+      <c r="BX6">
         <v>1.2</v>
       </c>
-      <c r="BX6">
+      <c r="BY6">
         <v>0.72</v>
       </c>
-      <c r="BY6">
+      <c r="BZ6">
         <v>0.73</v>
       </c>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7">
+        <v>0.99</v>
+      </c>
+      <c r="C7">
         <v>0.87</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>0.35</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.31</v>
       </c>
       <c r="E7" s="2">
         <v>0.31</v>
@@ -2617,125 +2637,125 @@
         <v>0.31</v>
       </c>
       <c r="G7" s="2">
+        <v>0.31</v>
+      </c>
+      <c r="H7" s="2">
         <v>0.13</v>
       </c>
-      <c r="H7" s="2">
+      <c r="I7" s="2">
         <v>0.05</v>
       </c>
-      <c r="I7" s="2">
+      <c r="J7" s="2">
         <v>-1.0900000000000001</v>
       </c>
-      <c r="J7" s="2">
+      <c r="K7" s="2">
         <v>-1.24</v>
       </c>
-      <c r="K7" s="2">
+      <c r="L7" s="2">
         <v>-1.21</v>
       </c>
-      <c r="L7" s="2">
+      <c r="M7" s="2">
         <v>-1.26</v>
       </c>
-      <c r="M7" s="2">
+      <c r="N7" s="2">
         <v>-1.21</v>
       </c>
-      <c r="N7" s="2">
+      <c r="O7" s="2">
         <v>-1.59</v>
       </c>
-      <c r="O7" s="2">
+      <c r="P7" s="2">
         <v>-1.57</v>
       </c>
-      <c r="P7" s="2">
+      <c r="Q7" s="2">
         <v>-0.79</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="R7" s="2">
         <v>-0.8</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>-0.8</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <v>-0.66</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>-0.64</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <v>-0.61</v>
       </c>
-      <c r="V7">
+      <c r="W7">
         <v>-0.28999999999999998</v>
-      </c>
-      <c r="W7">
-        <v>-0.48</v>
       </c>
       <c r="X7">
         <v>-0.48</v>
       </c>
       <c r="Y7">
+        <v>-0.48</v>
+      </c>
+      <c r="Z7">
         <v>-0.44</v>
       </c>
-      <c r="Z7">
+      <c r="AA7">
         <v>-0.3</v>
       </c>
-      <c r="AA7">
+      <c r="AB7">
         <v>-0.01</v>
       </c>
-      <c r="AB7">
+      <c r="AC7">
         <v>-0.44</v>
-      </c>
-      <c r="AC7">
-        <v>-0.31</v>
       </c>
       <c r="AD7">
         <v>-0.31</v>
       </c>
       <c r="AE7">
+        <v>-0.31</v>
+      </c>
+      <c r="AF7">
         <v>-0.3</v>
       </c>
-      <c r="AF7">
+      <c r="AG7">
         <v>-0.28999999999999998</v>
       </c>
-      <c r="AG7">
+      <c r="AH7">
         <v>-0.28000000000000003</v>
       </c>
-      <c r="AH7">
+      <c r="AI7">
         <v>-0.23</v>
       </c>
-      <c r="AI7">
+      <c r="AJ7">
         <v>-0.42</v>
       </c>
-      <c r="AJ7">
+      <c r="AK7">
         <v>-1.1499999999999999</v>
       </c>
-      <c r="AK7">
+      <c r="AL7">
         <v>-1.1599999999999999</v>
       </c>
-      <c r="AL7">
+      <c r="AM7">
         <v>-1.03</v>
       </c>
-      <c r="AM7">
+      <c r="AN7">
         <v>-1.5</v>
       </c>
-      <c r="AN7">
+      <c r="AO7">
         <v>-1.74</v>
       </c>
-      <c r="AO7">
+      <c r="AP7">
         <v>-1.83</v>
       </c>
-      <c r="AP7">
+      <c r="AQ7">
         <v>-1.27</v>
       </c>
-      <c r="AQ7">
+      <c r="AR7">
         <v>-1.24</v>
       </c>
-      <c r="AR7">
+      <c r="AS7">
         <v>-1.25</v>
       </c>
-      <c r="AS7">
+      <c r="AT7">
         <v>-1.27</v>
       </c>
-      <c r="AT7">
-        <v>0</v>
-      </c>
       <c r="AU7">
         <v>0</v>
       </c>
@@ -2812,163 +2832,166 @@
         <v>0</v>
       </c>
       <c r="BT7">
+        <v>0</v>
+      </c>
+      <c r="BU7">
         <v>-0.69</v>
       </c>
-      <c r="BU7">
+      <c r="BV7">
         <v>-0.67</v>
       </c>
-      <c r="BV7">
+      <c r="BW7">
         <v>-0.5</v>
       </c>
-      <c r="BW7">
+      <c r="BX7">
         <v>-0.56999999999999995</v>
       </c>
-      <c r="BX7">
+      <c r="BY7">
         <v>-1.25</v>
       </c>
-      <c r="BY7">
+      <c r="BZ7">
         <v>-0.73</v>
       </c>
     </row>
-    <row r="8" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8">
+        <v>-0.21</v>
+      </c>
+      <c r="C8">
         <v>-0.32</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>-1.08</v>
-      </c>
-      <c r="D8" s="2">
-        <v>-0.82</v>
       </c>
       <c r="E8" s="2">
         <v>-0.82</v>
       </c>
       <c r="F8" s="2">
+        <v>-0.82</v>
+      </c>
+      <c r="G8" s="2">
         <v>-0.81</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="2">
         <v>-0.95</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>-1.24</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J8" s="2">
         <v>-2.08</v>
-      </c>
-      <c r="J8" s="2">
-        <v>-1.89</v>
       </c>
       <c r="K8" s="2">
         <v>-1.89</v>
       </c>
       <c r="L8" s="2">
+        <v>-1.89</v>
+      </c>
+      <c r="M8" s="2">
         <v>-1.98</v>
       </c>
-      <c r="M8" s="2">
+      <c r="N8" s="2">
         <v>-1.94</v>
       </c>
-      <c r="N8" s="2">
+      <c r="O8" s="2">
         <v>-1.9</v>
       </c>
-      <c r="O8" s="2">
+      <c r="P8" s="2">
         <v>-1.48</v>
-      </c>
-      <c r="P8" s="2">
-        <v>-1.24</v>
       </c>
       <c r="Q8" s="2">
         <v>-1.24</v>
       </c>
-      <c r="R8">
+      <c r="R8" s="2">
         <v>-1.24</v>
       </c>
       <c r="S8">
-        <v>-1.06</v>
+        <v>-1.24</v>
       </c>
       <c r="T8">
         <v>-1.06</v>
       </c>
       <c r="U8">
+        <v>-1.06</v>
+      </c>
+      <c r="V8">
         <v>-1.22</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <v>-1.01</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <v>-0.73</v>
       </c>
-      <c r="Y8">
+      <c r="Z8">
         <v>-0.72</v>
       </c>
-      <c r="Z8">
+      <c r="AA8">
         <v>-0.99</v>
       </c>
-      <c r="AA8">
+      <c r="AB8">
         <v>-0.74</v>
       </c>
-      <c r="AB8">
+      <c r="AC8">
         <v>-0.85</v>
       </c>
-      <c r="AC8">
+      <c r="AD8">
         <v>-0.57999999999999996</v>
-      </c>
-      <c r="AD8">
-        <v>-0.56999999999999995</v>
       </c>
       <c r="AE8">
         <v>-0.56999999999999995</v>
       </c>
       <c r="AF8">
+        <v>-0.56999999999999995</v>
+      </c>
+      <c r="AG8">
         <v>-0.56000000000000005</v>
       </c>
-      <c r="AG8">
+      <c r="AH8">
         <v>-0.46</v>
       </c>
-      <c r="AH8">
+      <c r="AI8">
         <v>-0.51</v>
       </c>
-      <c r="AI8">
+      <c r="AJ8">
         <v>-0.8</v>
       </c>
-      <c r="AJ8">
+      <c r="AK8">
         <v>-1.64</v>
       </c>
-      <c r="AK8">
+      <c r="AL8">
         <v>-1.61</v>
       </c>
-      <c r="AL8">
+      <c r="AM8">
         <v>-1.39</v>
       </c>
-      <c r="AM8">
+      <c r="AN8">
         <v>-1.68</v>
       </c>
-      <c r="AN8">
+      <c r="AO8">
         <v>-1.93</v>
       </c>
-      <c r="AO8">
+      <c r="AP8">
         <v>-2.31</v>
       </c>
-      <c r="AP8">
+      <c r="AQ8">
         <v>-1.97</v>
       </c>
-      <c r="AQ8">
+      <c r="AR8">
         <v>-1.95</v>
       </c>
-      <c r="AR8">
+      <c r="AS8">
         <v>-1.94</v>
       </c>
-      <c r="AS8">
+      <c r="AT8">
         <v>-1.96</v>
       </c>
-      <c r="AT8">
-        <v>0</v>
-      </c>
       <c r="AU8">
         <v>0</v>
       </c>
@@ -3045,163 +3068,166 @@
         <v>0</v>
       </c>
       <c r="BT8">
+        <v>0</v>
+      </c>
+      <c r="BU8">
         <v>-0.78</v>
       </c>
-      <c r="BU8">
+      <c r="BV8">
         <v>-0.56999999999999995</v>
       </c>
-      <c r="BV8">
+      <c r="BW8">
         <v>-0.46</v>
       </c>
-      <c r="BW8">
+      <c r="BX8">
         <v>-0.5</v>
       </c>
-      <c r="BX8">
+      <c r="BY8">
         <v>-1.19</v>
       </c>
-      <c r="BY8">
+      <c r="BZ8">
         <v>-0.77</v>
       </c>
     </row>
-    <row r="9" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9">
+        <v>-0.17</v>
+      </c>
+      <c r="C9">
         <v>-0.08</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>-0.67</v>
-      </c>
-      <c r="D9" s="2">
-        <v>-0.66</v>
       </c>
       <c r="E9" s="2">
         <v>-0.66</v>
       </c>
       <c r="F9" s="2">
+        <v>-0.66</v>
+      </c>
+      <c r="G9" s="2">
         <v>-0.65</v>
       </c>
-      <c r="G9" s="2">
+      <c r="H9" s="2">
         <v>-0.89</v>
       </c>
-      <c r="H9" s="2">
+      <c r="I9" s="2">
         <v>-0.92</v>
       </c>
-      <c r="I9" s="2">
+      <c r="J9" s="2">
         <v>-1.78</v>
       </c>
-      <c r="J9" s="2">
+      <c r="K9" s="2">
         <v>-1.31</v>
       </c>
-      <c r="K9" s="2">
+      <c r="L9" s="2">
         <v>-1.28</v>
       </c>
-      <c r="L9" s="2">
+      <c r="M9" s="2">
         <v>-1.34</v>
       </c>
-      <c r="M9" s="2">
+      <c r="N9" s="2">
         <v>-1.38</v>
       </c>
-      <c r="N9" s="2">
+      <c r="O9" s="2">
         <v>-1.69</v>
       </c>
-      <c r="O9" s="2">
+      <c r="P9" s="2">
         <v>-1.37</v>
       </c>
-      <c r="P9" s="2">
+      <c r="Q9" s="2">
         <v>-1.1599999999999999</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="R9" s="2">
         <v>-1.17</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>-1.1599999999999999</v>
       </c>
-      <c r="S9">
+      <c r="T9">
         <v>-0.86</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>-0.85</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <v>-0.88</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <v>-1.18</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>-1.32</v>
       </c>
-      <c r="X9">
+      <c r="Y9">
         <v>-0.94</v>
       </c>
-      <c r="Y9">
+      <c r="Z9">
         <v>-0.87</v>
       </c>
-      <c r="Z9">
+      <c r="AA9">
         <v>-0.8</v>
       </c>
-      <c r="AA9">
+      <c r="AB9">
         <v>-0.53</v>
       </c>
-      <c r="AB9">
+      <c r="AC9">
         <v>-0.45</v>
-      </c>
-      <c r="AC9">
-        <v>-0.31</v>
       </c>
       <c r="AD9">
         <v>-0.31</v>
       </c>
       <c r="AE9">
-        <v>-0.3</v>
+        <v>-0.31</v>
       </c>
       <c r="AF9">
         <v>-0.3</v>
       </c>
       <c r="AG9">
-        <v>-0.28000000000000003</v>
+        <v>-0.3</v>
       </c>
       <c r="AH9">
         <v>-0.28000000000000003</v>
       </c>
       <c r="AI9">
+        <v>-0.28000000000000003</v>
+      </c>
+      <c r="AJ9">
         <v>-0.51</v>
       </c>
-      <c r="AJ9">
+      <c r="AK9">
         <v>-1.22</v>
       </c>
-      <c r="AK9">
+      <c r="AL9">
         <v>-1.24</v>
       </c>
-      <c r="AL9">
+      <c r="AM9">
         <v>-1.2</v>
       </c>
-      <c r="AM9">
+      <c r="AN9">
         <v>-1.43</v>
       </c>
-      <c r="AN9">
+      <c r="AO9">
         <v>-1.76</v>
       </c>
-      <c r="AO9">
+      <c r="AP9">
         <v>-1.92</v>
       </c>
-      <c r="AP9">
+      <c r="AQ9">
         <v>-1.27</v>
       </c>
-      <c r="AQ9">
+      <c r="AR9">
         <v>-1.26</v>
       </c>
-      <c r="AR9">
+      <c r="AS9">
         <v>-1.25</v>
       </c>
-      <c r="AS9">
+      <c r="AT9">
         <v>-1.27</v>
       </c>
-      <c r="AT9">
-        <v>0</v>
-      </c>
       <c r="AU9">
         <v>0</v>
       </c>
@@ -3278,163 +3304,166 @@
         <v>0</v>
       </c>
       <c r="BT9">
+        <v>0</v>
+      </c>
+      <c r="BU9">
         <v>-0.76</v>
       </c>
-      <c r="BU9">
+      <c r="BV9">
         <v>-0.59</v>
       </c>
-      <c r="BV9">
+      <c r="BW9">
         <v>-0.49</v>
       </c>
-      <c r="BW9">
+      <c r="BX9">
         <v>-0.61</v>
       </c>
-      <c r="BX9">
+      <c r="BY9">
         <v>-1.75</v>
       </c>
-      <c r="BY9">
+      <c r="BZ9">
         <v>-1.5</v>
       </c>
     </row>
-    <row r="10" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>101</v>
       </c>
       <c r="B10">
+        <v>-0.3</v>
+      </c>
+      <c r="C10">
         <v>-0.19</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>-0.72</v>
       </c>
-      <c r="D10" s="2">
+      <c r="E10" s="2">
         <v>-0.73</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>-0.72</v>
-      </c>
-      <c r="F10" s="2">
-        <v>-0.71</v>
       </c>
       <c r="G10" s="2">
         <v>-0.71</v>
       </c>
       <c r="H10" s="2">
+        <v>-0.71</v>
+      </c>
+      <c r="I10" s="2">
         <v>-0.65</v>
       </c>
-      <c r="I10" s="2">
+      <c r="J10" s="2">
         <v>-1.21</v>
       </c>
-      <c r="J10" s="2">
+      <c r="K10" s="2">
         <v>-1.0900000000000001</v>
       </c>
-      <c r="K10" s="2">
+      <c r="L10" s="2">
         <v>-1.08</v>
       </c>
-      <c r="L10" s="2">
+      <c r="M10" s="2">
         <v>-1.1499999999999999</v>
       </c>
-      <c r="M10" s="2">
+      <c r="N10" s="2">
         <v>-1.1200000000000001</v>
       </c>
-      <c r="N10" s="2">
+      <c r="O10" s="2">
         <v>-1.58</v>
       </c>
-      <c r="O10" s="2">
+      <c r="P10" s="2">
         <v>-1.07</v>
       </c>
-      <c r="P10" s="2">
+      <c r="Q10" s="2">
         <v>-0.32</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="R10" s="2">
         <v>-0.33</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>-0.33</v>
-      </c>
-      <c r="S10">
-        <v>-0.25</v>
       </c>
       <c r="T10">
         <v>-0.25</v>
       </c>
       <c r="U10">
+        <v>-0.25</v>
+      </c>
+      <c r="V10">
         <v>-0.28999999999999998</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <v>-0.13</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>-0.26</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <v>-1.1200000000000001</v>
       </c>
-      <c r="Y10">
+      <c r="Z10">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="Z10">
+      <c r="AA10">
         <v>-1</v>
       </c>
-      <c r="AA10">
+      <c r="AB10">
         <v>-0.73</v>
       </c>
-      <c r="AB10">
+      <c r="AC10">
         <v>-1.45</v>
       </c>
-      <c r="AC10">
+      <c r="AD10">
         <v>-1.3</v>
       </c>
-      <c r="AD10">
+      <c r="AE10">
         <v>-1.29</v>
-      </c>
-      <c r="AE10">
-        <v>-1.28</v>
       </c>
       <c r="AF10">
         <v>-1.28</v>
       </c>
       <c r="AG10">
+        <v>-1.28</v>
+      </c>
+      <c r="AH10">
         <v>-1.27</v>
       </c>
-      <c r="AH10">
+      <c r="AI10">
         <v>-1.28</v>
       </c>
-      <c r="AI10">
+      <c r="AJ10">
         <v>-1.75</v>
       </c>
-      <c r="AJ10">
+      <c r="AK10">
         <v>-1.92</v>
       </c>
-      <c r="AK10">
+      <c r="AL10">
         <v>-1.91</v>
       </c>
-      <c r="AL10">
+      <c r="AM10">
         <v>-1.87</v>
       </c>
-      <c r="AM10">
+      <c r="AN10">
         <v>-2.41</v>
       </c>
-      <c r="AN10">
+      <c r="AO10">
         <v>-2.4300000000000002</v>
       </c>
-      <c r="AO10">
+      <c r="AP10">
         <v>-2.65</v>
       </c>
-      <c r="AP10">
+      <c r="AQ10">
         <v>-2.21</v>
       </c>
-      <c r="AQ10">
+      <c r="AR10">
         <v>-2.1800000000000002</v>
       </c>
-      <c r="AR10">
+      <c r="AS10">
         <v>-2.19</v>
       </c>
-      <c r="AS10">
+      <c r="AT10">
         <v>-2.2200000000000002</v>
       </c>
-      <c r="AT10">
-        <v>0</v>
-      </c>
       <c r="AU10">
         <v>0</v>
       </c>
@@ -3511,163 +3540,166 @@
         <v>0</v>
       </c>
       <c r="BT10">
+        <v>0</v>
+      </c>
+      <c r="BU10">
         <v>-0.2</v>
       </c>
-      <c r="BU10">
+      <c r="BV10">
         <v>-0.38</v>
       </c>
-      <c r="BV10">
+      <c r="BW10">
         <v>-0.33</v>
       </c>
-      <c r="BW10">
+      <c r="BX10">
         <v>-0.45</v>
       </c>
-      <c r="BX10">
+      <c r="BY10">
         <v>-1.05</v>
       </c>
-      <c r="BY10">
+      <c r="BZ10">
         <v>-0.53</v>
       </c>
     </row>
-    <row r="11" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
       <c r="B11">
+        <v>0.26</v>
+      </c>
+      <c r="C11">
         <v>-0.25</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>-0.3</v>
       </c>
-      <c r="D11" s="2">
+      <c r="E11" s="2">
         <v>-0.32</v>
-      </c>
-      <c r="E11" s="2">
-        <v>-0.33</v>
       </c>
       <c r="F11" s="2">
         <v>-0.33</v>
       </c>
       <c r="G11" s="2">
+        <v>-0.33</v>
+      </c>
+      <c r="H11" s="2">
         <v>-0.05</v>
       </c>
-      <c r="H11" s="2">
+      <c r="I11" s="2">
         <v>-0.14000000000000001</v>
       </c>
-      <c r="I11" s="2">
+      <c r="J11" s="2">
         <v>0.15</v>
       </c>
-      <c r="J11" s="2">
+      <c r="K11" s="2">
         <v>-0.65</v>
       </c>
-      <c r="K11" s="2">
+      <c r="L11" s="2">
         <v>-0.63</v>
       </c>
-      <c r="L11" s="2">
+      <c r="M11" s="2">
         <v>-0.74</v>
       </c>
-      <c r="M11" s="2">
+      <c r="N11" s="2">
         <v>-0.73</v>
       </c>
-      <c r="N11" s="2">
+      <c r="O11" s="2">
         <v>-0.91</v>
-      </c>
-      <c r="O11" s="2">
-        <v>-0.51</v>
       </c>
       <c r="P11" s="2">
         <v>-0.51</v>
       </c>
       <c r="Q11" s="2">
+        <v>-0.51</v>
+      </c>
+      <c r="R11" s="2">
         <v>-0.52</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>-0.51</v>
-      </c>
-      <c r="S11">
-        <v>-0.85</v>
       </c>
       <c r="T11">
         <v>-0.85</v>
       </c>
       <c r="U11">
+        <v>-0.85</v>
+      </c>
+      <c r="V11">
         <v>-1.26</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <v>-0.86</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <v>-0.77</v>
       </c>
-      <c r="X11">
+      <c r="Y11">
         <v>-1.08</v>
       </c>
-      <c r="Y11">
+      <c r="Z11">
         <v>-1.01</v>
       </c>
-      <c r="Z11">
+      <c r="AA11">
         <v>-1.1100000000000001</v>
       </c>
-      <c r="AA11">
+      <c r="AB11">
         <v>-0.98</v>
       </c>
-      <c r="AB11">
+      <c r="AC11">
         <v>-0.49</v>
       </c>
-      <c r="AC11">
+      <c r="AD11">
         <v>-0.2</v>
       </c>
-      <c r="AD11">
+      <c r="AE11">
         <v>-0.19</v>
       </c>
-      <c r="AE11">
+      <c r="AF11">
         <v>-0.2</v>
       </c>
-      <c r="AF11">
+      <c r="AG11">
         <v>-0.19</v>
       </c>
-      <c r="AG11">
-        <v>0</v>
-      </c>
       <c r="AH11">
+        <v>0</v>
+      </c>
+      <c r="AI11">
         <v>0.12</v>
       </c>
-      <c r="AI11">
+      <c r="AJ11">
         <v>-0.28000000000000003</v>
       </c>
-      <c r="AJ11">
+      <c r="AK11">
         <v>-0.27</v>
       </c>
-      <c r="AK11">
+      <c r="AL11">
         <v>-0.28000000000000003</v>
       </c>
-      <c r="AL11">
+      <c r="AM11">
         <v>-0.12</v>
       </c>
-      <c r="AM11">
+      <c r="AN11">
         <v>-0.37</v>
       </c>
-      <c r="AN11">
+      <c r="AO11">
         <v>-1.54</v>
       </c>
-      <c r="AO11">
+      <c r="AP11">
         <v>-1.82</v>
       </c>
-      <c r="AP11">
+      <c r="AQ11">
         <v>-1.48</v>
       </c>
-      <c r="AQ11">
+      <c r="AR11">
         <v>-1.5</v>
       </c>
-      <c r="AR11">
+      <c r="AS11">
         <v>-1.49</v>
       </c>
-      <c r="AS11">
+      <c r="AT11">
         <v>-1.48</v>
       </c>
-      <c r="AT11">
-        <v>0</v>
-      </c>
       <c r="AU11">
         <v>0</v>
       </c>
@@ -3744,163 +3776,166 @@
         <v>0</v>
       </c>
       <c r="BT11">
+        <v>0</v>
+      </c>
+      <c r="BU11">
         <v>-1.22</v>
       </c>
-      <c r="BU11">
+      <c r="BV11">
         <v>-0.89</v>
       </c>
-      <c r="BV11">
+      <c r="BW11">
         <v>-0.81</v>
       </c>
-      <c r="BW11">
+      <c r="BX11">
         <v>-1.01</v>
       </c>
-      <c r="BX11">
+      <c r="BY11">
         <v>-1.94</v>
       </c>
-      <c r="BY11">
+      <c r="BZ11">
         <v>-1.26</v>
       </c>
     </row>
-    <row r="12" spans="1:78" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:79" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>9</v>
       </c>
       <c r="B12">
+        <v>1.91</v>
+      </c>
+      <c r="C12">
         <v>1.83</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>1.22</v>
       </c>
-      <c r="D12" s="2">
+      <c r="E12" s="2">
         <v>1.02</v>
-      </c>
-      <c r="E12" s="2">
-        <v>1.03</v>
       </c>
       <c r="F12" s="2">
         <v>1.03</v>
       </c>
       <c r="G12" s="2">
+        <v>1.03</v>
+      </c>
+      <c r="H12" s="2">
         <v>0.53</v>
       </c>
-      <c r="H12" s="2">
+      <c r="I12" s="2">
         <v>0.22</v>
       </c>
-      <c r="I12" s="2">
+      <c r="J12" s="2">
         <v>-0.49</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0.33</v>
       </c>
       <c r="K12" s="2">
         <v>0.33</v>
       </c>
       <c r="L12" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="M12" s="2">
         <v>0.04</v>
       </c>
-      <c r="M12" s="2">
+      <c r="N12" s="2">
         <v>0.05</v>
       </c>
-      <c r="N12" s="2">
+      <c r="O12" s="2">
         <v>0.09</v>
       </c>
-      <c r="O12" s="2">
+      <c r="P12" s="2">
         <v>0.3</v>
       </c>
-      <c r="P12" s="2">
+      <c r="Q12" s="2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="R12" s="2">
         <v>0.13</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>0.14000000000000001</v>
       </c>
-      <c r="S12">
+      <c r="T12">
         <v>0.71</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <v>0.72</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <v>0.93</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <v>-0.34</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <v>-0.96</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <v>-1.56</v>
       </c>
-      <c r="Y12">
+      <c r="Z12">
         <v>-1.61</v>
       </c>
-      <c r="Z12">
+      <c r="AA12">
         <v>-1.56</v>
       </c>
-      <c r="AA12">
+      <c r="AB12">
         <v>-1.1299999999999999</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
         <v>-1.03</v>
       </c>
-      <c r="AC12">
+      <c r="AD12">
         <v>-0.81</v>
       </c>
-      <c r="AD12">
+      <c r="AE12">
         <v>-0.79</v>
       </c>
-      <c r="AE12">
+      <c r="AF12">
         <v>-0.77</v>
       </c>
-      <c r="AF12">
+      <c r="AG12">
         <v>-0.78</v>
       </c>
-      <c r="AG12">
+      <c r="AH12">
         <v>-0.98</v>
       </c>
-      <c r="AH12">
+      <c r="AI12">
         <v>-0.67</v>
-      </c>
-      <c r="AI12">
-        <v>-0.59</v>
       </c>
       <c r="AJ12">
         <v>-0.59</v>
       </c>
       <c r="AK12">
+        <v>-0.59</v>
+      </c>
+      <c r="AL12">
         <v>-0.51</v>
       </c>
-      <c r="AL12">
+      <c r="AM12">
         <v>-0.63</v>
       </c>
-      <c r="AM12">
+      <c r="AN12">
         <v>-1.17</v>
       </c>
-      <c r="AN12">
+      <c r="AO12">
         <v>-1.53</v>
       </c>
-      <c r="AO12">
+      <c r="AP12">
         <v>-1.78</v>
-      </c>
-      <c r="AP12">
-        <v>-1.19</v>
       </c>
       <c r="AQ12">
         <v>-1.19</v>
       </c>
       <c r="AR12">
+        <v>-1.19</v>
+      </c>
+      <c r="AS12">
         <v>-1.18</v>
       </c>
-      <c r="AS12">
+      <c r="AT12">
         <v>-1.2</v>
       </c>
-      <c r="AT12">
-        <v>0</v>
-      </c>
       <c r="AU12">
         <v>0</v>
       </c>
@@ -3977,163 +4012,166 @@
         <v>0</v>
       </c>
       <c r="BT12">
+        <v>0</v>
+      </c>
+      <c r="BU12">
         <v>-0.15</v>
       </c>
-      <c r="BU12">
+      <c r="BV12">
         <v>-0.49</v>
       </c>
-      <c r="BV12">
+      <c r="BW12">
         <v>-0.35</v>
       </c>
-      <c r="BW12">
+      <c r="BX12">
         <v>-0.45</v>
       </c>
-      <c r="BX12">
+      <c r="BY12">
         <v>-1.37</v>
       </c>
-      <c r="BY12">
+      <c r="BZ12">
         <v>-1.03</v>
       </c>
     </row>
-    <row r="13" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
       <c r="B13">
+        <v>0.45</v>
+      </c>
+      <c r="C13">
         <v>0.27</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>-7.0000000000000007E-2</v>
       </c>
-      <c r="D13" s="2">
+      <c r="E13" s="2">
         <v>0.23</v>
-      </c>
-      <c r="E13" s="2">
-        <v>0.22</v>
       </c>
       <c r="F13" s="2">
         <v>0.22</v>
       </c>
       <c r="G13" s="2">
+        <v>0.22</v>
+      </c>
+      <c r="H13" s="2">
         <v>-0.05</v>
       </c>
-      <c r="H13" s="2">
+      <c r="I13" s="2">
         <v>-0.28999999999999998</v>
       </c>
-      <c r="I13" s="2">
+      <c r="J13" s="2">
         <v>-1.1299999999999999</v>
       </c>
-      <c r="J13" s="2">
+      <c r="K13" s="2">
         <v>-1.2</v>
       </c>
-      <c r="K13" s="2">
+      <c r="L13" s="2">
         <v>-1.17</v>
       </c>
-      <c r="L13" s="2">
+      <c r="M13" s="2">
         <v>-0.92</v>
       </c>
-      <c r="M13" s="2">
+      <c r="N13" s="2">
         <v>-0.91</v>
       </c>
-      <c r="N13" s="2">
+      <c r="O13" s="2">
         <v>-0.78</v>
       </c>
-      <c r="O13" s="2">
+      <c r="P13" s="2">
         <v>-0.85</v>
-      </c>
-      <c r="P13" s="2">
-        <v>-0.79</v>
       </c>
       <c r="Q13" s="2">
         <v>-0.79</v>
       </c>
-      <c r="R13">
+      <c r="R13" s="2">
         <v>-0.79</v>
       </c>
       <c r="S13">
+        <v>-0.79</v>
+      </c>
+      <c r="T13">
         <v>-0.5</v>
       </c>
-      <c r="T13">
+      <c r="U13">
         <v>-0.49</v>
       </c>
-      <c r="U13">
+      <c r="V13">
         <v>-0.64</v>
       </c>
-      <c r="V13">
+      <c r="W13">
         <v>-0.1</v>
       </c>
-      <c r="W13">
+      <c r="X13">
         <v>-0.45</v>
       </c>
-      <c r="X13">
+      <c r="Y13">
         <v>-1.1599999999999999</v>
       </c>
-      <c r="Y13">
+      <c r="Z13">
         <v>-1.18</v>
       </c>
-      <c r="Z13">
+      <c r="AA13">
         <v>-1.17</v>
       </c>
-      <c r="AA13">
+      <c r="AB13">
         <v>-1.01</v>
       </c>
-      <c r="AB13">
+      <c r="AC13">
         <v>-0.89</v>
       </c>
-      <c r="AC13">
+      <c r="AD13">
         <v>-0.77</v>
       </c>
-      <c r="AD13">
+      <c r="AE13">
         <v>-0.76</v>
       </c>
-      <c r="AE13">
+      <c r="AF13">
         <v>-0.75</v>
       </c>
-      <c r="AF13">
+      <c r="AG13">
         <v>-0.78</v>
       </c>
-      <c r="AG13">
+      <c r="AH13">
         <v>-0.69</v>
       </c>
-      <c r="AH13">
+      <c r="AI13">
         <v>-0.83</v>
       </c>
-      <c r="AI13">
+      <c r="AJ13">
         <v>-1.38</v>
       </c>
-      <c r="AJ13">
+      <c r="AK13">
         <v>-1.43</v>
       </c>
-      <c r="AK13">
+      <c r="AL13">
         <v>-1.39</v>
       </c>
-      <c r="AL13">
+      <c r="AM13">
         <v>-1.48</v>
       </c>
-      <c r="AM13">
+      <c r="AN13">
         <v>-1.99</v>
       </c>
-      <c r="AN13">
+      <c r="AO13">
         <v>-2.2400000000000002</v>
       </c>
-      <c r="AO13">
+      <c r="AP13">
         <v>-2.36</v>
       </c>
-      <c r="AP13">
+      <c r="AQ13">
         <v>-1.23</v>
       </c>
-      <c r="AQ13">
+      <c r="AR13">
         <v>-1.2</v>
       </c>
-      <c r="AR13">
+      <c r="AS13">
         <v>-1.19</v>
       </c>
-      <c r="AS13">
+      <c r="AT13">
         <v>-1.23</v>
       </c>
-      <c r="AT13">
-        <v>0</v>
-      </c>
       <c r="AU13">
         <v>0</v>
       </c>
@@ -4210,36 +4248,39 @@
         <v>0</v>
       </c>
       <c r="BT13">
+        <v>0</v>
+      </c>
+      <c r="BU13">
         <v>0.8</v>
       </c>
-      <c r="BU13">
+      <c r="BV13">
         <v>0.66</v>
       </c>
-      <c r="BV13">
+      <c r="BW13">
         <v>0.83</v>
       </c>
-      <c r="BW13">
+      <c r="BX13">
         <v>0.81</v>
       </c>
-      <c r="BX13">
+      <c r="BY13">
         <v>-0.41</v>
       </c>
-      <c r="BY13">
+      <c r="BZ13">
         <v>-0.48</v>
       </c>
     </row>
-    <row r="14" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
       <c r="B14">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="C14">
         <v>-0.15</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>-0.45</v>
-      </c>
-      <c r="D14" s="2">
-        <v>-0.44</v>
       </c>
       <c r="E14" s="2">
         <v>-0.44</v>
@@ -4248,125 +4289,125 @@
         <v>-0.44</v>
       </c>
       <c r="G14" s="2">
+        <v>-0.44</v>
+      </c>
+      <c r="H14" s="2">
         <v>-0.55000000000000004</v>
       </c>
-      <c r="H14" s="2">
+      <c r="I14" s="2">
         <v>-0.24</v>
       </c>
-      <c r="I14" s="2">
+      <c r="J14" s="2">
         <v>-1.04</v>
       </c>
-      <c r="J14" s="2">
+      <c r="K14" s="2">
         <v>-0.71</v>
       </c>
-      <c r="K14" s="2">
+      <c r="L14" s="2">
         <v>-0.7</v>
       </c>
-      <c r="L14" s="2">
+      <c r="M14" s="2">
         <v>-0.64</v>
       </c>
-      <c r="M14" s="2">
+      <c r="N14" s="2">
         <v>-0.63</v>
       </c>
-      <c r="N14" s="2">
+      <c r="O14" s="2">
         <v>-0.69</v>
       </c>
-      <c r="O14" s="2">
+      <c r="P14" s="2">
         <v>-0.95</v>
-      </c>
-      <c r="P14" s="2">
-        <v>-1.05</v>
       </c>
       <c r="Q14" s="2">
         <v>-1.05</v>
       </c>
-      <c r="R14">
+      <c r="R14" s="2">
+        <v>-1.05</v>
+      </c>
+      <c r="S14">
         <v>-1.04</v>
       </c>
-      <c r="S14">
+      <c r="T14">
         <v>-0.92</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>-0.91</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <v>-0.92</v>
       </c>
-      <c r="V14">
+      <c r="W14">
         <v>-1.39</v>
       </c>
-      <c r="W14">
+      <c r="X14">
         <v>-1.95</v>
       </c>
-      <c r="X14">
+      <c r="Y14">
         <v>-1.87</v>
       </c>
-      <c r="Y14">
+      <c r="Z14">
         <v>-1.84</v>
       </c>
-      <c r="Z14">
+      <c r="AA14">
         <v>-1.91</v>
       </c>
-      <c r="AA14">
+      <c r="AB14">
         <v>-1.47</v>
       </c>
-      <c r="AB14">
+      <c r="AC14">
         <v>-1.63</v>
       </c>
-      <c r="AC14">
+      <c r="AD14">
         <v>-1.38</v>
       </c>
-      <c r="AD14">
+      <c r="AE14">
         <v>-1.39</v>
       </c>
-      <c r="AE14">
+      <c r="AF14">
         <v>-1.37</v>
       </c>
-      <c r="AF14">
+      <c r="AG14">
         <v>-1.4</v>
       </c>
-      <c r="AG14">
+      <c r="AH14">
         <v>-1.41</v>
       </c>
-      <c r="AH14">
+      <c r="AI14">
         <v>-1.43</v>
       </c>
-      <c r="AI14">
+      <c r="AJ14">
         <v>-1.44</v>
       </c>
-      <c r="AJ14">
+      <c r="AK14">
         <v>-1.6</v>
       </c>
-      <c r="AK14">
+      <c r="AL14">
         <v>-1.62</v>
       </c>
-      <c r="AL14">
+      <c r="AM14">
         <v>-1.59</v>
       </c>
-      <c r="AM14">
+      <c r="AN14">
         <v>-1.94</v>
       </c>
-      <c r="AN14">
+      <c r="AO14">
         <v>-1.91</v>
       </c>
-      <c r="AO14">
+      <c r="AP14">
         <v>-2.1800000000000002</v>
       </c>
-      <c r="AP14">
+      <c r="AQ14">
         <v>-1.56</v>
-      </c>
-      <c r="AQ14">
-        <v>-1.55</v>
       </c>
       <c r="AR14">
         <v>-1.55</v>
       </c>
       <c r="AS14">
+        <v>-1.55</v>
+      </c>
+      <c r="AT14">
         <v>-1.56</v>
       </c>
-      <c r="AT14">
-        <v>0</v>
-      </c>
       <c r="AU14">
         <v>0</v>
       </c>
@@ -4443,163 +4484,166 @@
         <v>0</v>
       </c>
       <c r="BT14">
+        <v>0</v>
+      </c>
+      <c r="BU14">
         <v>-0.53</v>
       </c>
-      <c r="BU14">
+      <c r="BV14">
         <v>-0.28000000000000003</v>
       </c>
-      <c r="BV14">
+      <c r="BW14">
         <v>-0.31</v>
       </c>
-      <c r="BW14">
+      <c r="BX14">
         <v>-0.42</v>
       </c>
-      <c r="BX14">
+      <c r="BY14">
         <v>-1.41</v>
       </c>
-      <c r="BY14">
+      <c r="BZ14">
         <v>-0.81</v>
       </c>
     </row>
-    <row r="15" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
       <c r="B15">
+        <v>0.41</v>
+      </c>
+      <c r="C15">
         <v>0.34</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>-0.38</v>
-      </c>
-      <c r="D15" s="2">
-        <v>-0.26</v>
       </c>
       <c r="E15" s="2">
         <v>-0.26</v>
       </c>
       <c r="F15" s="2">
+        <v>-0.26</v>
+      </c>
+      <c r="G15" s="2">
         <v>-0.25</v>
       </c>
-      <c r="G15" s="2">
+      <c r="H15" s="2">
         <v>-0.42</v>
       </c>
-      <c r="H15" s="2">
+      <c r="I15" s="2">
         <v>-0.56000000000000005</v>
       </c>
-      <c r="I15" s="2">
+      <c r="J15" s="2">
         <v>-1.67</v>
       </c>
-      <c r="J15" s="2">
+      <c r="K15" s="2">
         <v>-1.44</v>
       </c>
-      <c r="K15" s="2">
+      <c r="L15" s="2">
         <v>-1.43</v>
       </c>
-      <c r="L15" s="2">
+      <c r="M15" s="2">
         <v>-1.4</v>
       </c>
-      <c r="M15" s="2">
+      <c r="N15" s="2">
         <v>-1.38</v>
       </c>
-      <c r="N15" s="2">
+      <c r="O15" s="2">
         <v>-1.52</v>
       </c>
-      <c r="O15" s="2">
+      <c r="P15" s="2">
         <v>-1.1499999999999999</v>
       </c>
-      <c r="P15" s="2">
+      <c r="Q15" s="2">
         <v>-0.79</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="R15" s="2">
         <v>-0.8</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>-0.79</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>-0.59</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <v>-0.76</v>
       </c>
-      <c r="V15">
+      <c r="W15">
         <v>-0.49</v>
       </c>
-      <c r="W15">
+      <c r="X15">
         <v>-0.61</v>
       </c>
-      <c r="X15">
+      <c r="Y15">
         <v>-0.9</v>
       </c>
-      <c r="Y15">
+      <c r="Z15">
         <v>-0.86</v>
       </c>
-      <c r="Z15">
+      <c r="AA15">
         <v>-0.95</v>
       </c>
-      <c r="AA15">
+      <c r="AB15">
         <v>-0.7</v>
       </c>
-      <c r="AB15">
+      <c r="AC15">
         <v>-0.78</v>
-      </c>
-      <c r="AC15">
-        <v>-0.64</v>
       </c>
       <c r="AD15">
         <v>-0.64</v>
       </c>
       <c r="AE15">
+        <v>-0.64</v>
+      </c>
+      <c r="AF15">
         <v>-0.63</v>
       </c>
-      <c r="AF15">
+      <c r="AG15">
         <v>-0.62</v>
       </c>
-      <c r="AG15">
+      <c r="AH15">
         <v>-0.53</v>
       </c>
-      <c r="AH15">
+      <c r="AI15">
         <v>-0.65</v>
       </c>
-      <c r="AI15">
+      <c r="AJ15">
         <v>-0.74</v>
       </c>
-      <c r="AJ15">
+      <c r="AK15">
         <v>-1.29</v>
       </c>
-      <c r="AK15">
+      <c r="AL15">
         <v>-1.3</v>
       </c>
-      <c r="AL15">
+      <c r="AM15">
         <v>-1.1100000000000001</v>
       </c>
-      <c r="AM15">
+      <c r="AN15">
         <v>-1.43</v>
       </c>
-      <c r="AN15">
+      <c r="AO15">
         <v>-1.83</v>
       </c>
-      <c r="AO15">
+      <c r="AP15">
         <v>-1.86</v>
       </c>
-      <c r="AP15">
+      <c r="AQ15">
         <v>-1.32</v>
-      </c>
-      <c r="AQ15">
-        <v>-1.31</v>
       </c>
       <c r="AR15">
         <v>-1.31</v>
       </c>
       <c r="AS15">
+        <v>-1.31</v>
+      </c>
+      <c r="AT15">
         <v>-1.33</v>
       </c>
-      <c r="AT15">
-        <v>0</v>
-      </c>
       <c r="AU15">
         <v>0</v>
       </c>
@@ -4676,114 +4720,117 @@
         <v>0</v>
       </c>
       <c r="BT15">
+        <v>0</v>
+      </c>
+      <c r="BU15">
         <v>-0.38</v>
       </c>
-      <c r="BU15">
+      <c r="BV15">
         <v>-0.21</v>
       </c>
-      <c r="BV15">
+      <c r="BW15">
         <v>-0.14000000000000001</v>
       </c>
-      <c r="BW15">
+      <c r="BX15">
         <v>-0.21</v>
       </c>
-      <c r="BX15">
+      <c r="BY15">
         <v>-1.03</v>
       </c>
-      <c r="BY15">
+      <c r="BZ15">
         <v>-0.67</v>
       </c>
     </row>
-    <row r="16" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
       <c r="B16">
+        <v>0.46</v>
+      </c>
+      <c r="C16">
         <v>0.39</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>-0.27</v>
-      </c>
-      <c r="D16" s="2">
-        <v>-0.22</v>
       </c>
       <c r="E16" s="2">
         <v>-0.22</v>
       </c>
       <c r="F16" s="2">
+        <v>-0.22</v>
+      </c>
+      <c r="G16" s="2">
         <v>-0.21</v>
       </c>
-      <c r="G16" s="2">
+      <c r="H16" s="2">
         <v>-0.37</v>
       </c>
-      <c r="H16" s="2">
+      <c r="I16" s="2">
         <v>-0.43</v>
       </c>
-      <c r="I16" s="2">
+      <c r="J16" s="2">
         <v>-1.55</v>
       </c>
-      <c r="J16" s="2">
+      <c r="K16" s="2">
         <v>-1.4</v>
       </c>
-      <c r="K16" s="2">
+      <c r="L16" s="2">
         <v>-1.38</v>
       </c>
-      <c r="L16" s="2">
+      <c r="M16" s="2">
         <v>-1.48</v>
       </c>
-      <c r="M16" s="2">
+      <c r="N16" s="2">
         <v>-1.45</v>
       </c>
-      <c r="N16" s="2">
+      <c r="O16" s="2">
         <v>-1.7</v>
       </c>
-      <c r="O16" s="2">
+      <c r="P16" s="2">
         <v>-1.44</v>
       </c>
-      <c r="P16" s="2">
+      <c r="Q16" s="2">
         <v>-1.0900000000000001</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="R16" s="2">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="R16">
+      <c r="S16">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="S16">
+      <c r="T16">
         <v>-0.95</v>
       </c>
-      <c r="T16">
+      <c r="U16">
         <v>-0.94</v>
       </c>
-      <c r="U16">
+      <c r="V16">
         <v>-1</v>
       </c>
-      <c r="V16">
+      <c r="W16">
         <v>-1.08</v>
       </c>
-      <c r="W16">
+      <c r="X16">
         <v>-1.27</v>
       </c>
-      <c r="X16">
+      <c r="Y16">
         <v>-1.1000000000000001</v>
       </c>
-      <c r="Y16">
+      <c r="Z16">
         <v>-1.07</v>
       </c>
-      <c r="Z16">
+      <c r="AA16">
         <v>-1.02</v>
       </c>
-      <c r="AA16">
+      <c r="AB16">
         <v>-0.71</v>
       </c>
-      <c r="AB16">
+      <c r="AC16">
         <v>-0.85</v>
       </c>
-      <c r="AC16">
+      <c r="AD16">
         <v>-0.65</v>
-      </c>
-      <c r="AD16">
-        <v>-0.64</v>
       </c>
       <c r="AE16">
         <v>-0.64</v>
@@ -4792,153 +4839,156 @@
         <v>-0.64</v>
       </c>
       <c r="AG16">
+        <v>-0.64</v>
+      </c>
+      <c r="AH16">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="AH16">
+      <c r="AI16">
         <v>-0.53</v>
       </c>
-      <c r="AI16">
+      <c r="AJ16">
         <v>-0.92</v>
       </c>
-      <c r="AJ16">
+      <c r="AK16">
         <v>-1.58</v>
       </c>
-      <c r="AK16">
+      <c r="AL16">
         <v>-1.57</v>
       </c>
-      <c r="AL16">
+      <c r="AM16">
         <v>-1.51</v>
       </c>
-      <c r="AM16">
+      <c r="AN16">
         <v>-1.9</v>
       </c>
-      <c r="AN16">
+      <c r="AO16">
         <v>-2.17</v>
       </c>
-      <c r="AO16">
+      <c r="AP16">
         <v>-2.39</v>
       </c>
-      <c r="AP16">
+      <c r="AQ16">
         <v>-1.9</v>
       </c>
-      <c r="AQ16">
+      <c r="AR16">
         <v>-1.86</v>
-      </c>
-      <c r="AR16">
-        <v>-1.85</v>
       </c>
       <c r="AS16">
         <v>-1.85</v>
       </c>
       <c r="AT16">
-        <v>-1.89</v>
+        <v>-1.85</v>
       </c>
       <c r="AU16">
         <v>-1.89</v>
       </c>
       <c r="AV16">
+        <v>-1.89</v>
+      </c>
+      <c r="AW16">
         <v>-1.32</v>
       </c>
-      <c r="AW16">
+      <c r="AX16">
         <v>-1.3</v>
       </c>
-      <c r="AX16">
+      <c r="AY16">
         <v>-1.28</v>
       </c>
-      <c r="AY16">
+      <c r="AZ16">
         <v>-1.2</v>
       </c>
-      <c r="AZ16">
+      <c r="BA16">
         <v>-0.82</v>
       </c>
-      <c r="BA16">
+      <c r="BB16">
         <v>-0.97</v>
       </c>
-      <c r="BB16">
+      <c r="BC16">
         <v>-1.01</v>
       </c>
-      <c r="BC16">
+      <c r="BD16">
         <v>-1.03</v>
       </c>
-      <c r="BD16">
+      <c r="BE16">
         <v>-1.1299999999999999</v>
       </c>
-      <c r="BE16">
+      <c r="BF16">
         <v>-1.36</v>
       </c>
-      <c r="BF16">
+      <c r="BG16">
         <v>-1.1399999999999999</v>
       </c>
-      <c r="BG16">
+      <c r="BH16">
         <v>-1.1200000000000001</v>
       </c>
-      <c r="BH16">
+      <c r="BI16">
         <v>-1.1100000000000001</v>
       </c>
-      <c r="BI16">
+      <c r="BJ16">
         <v>-1.1000000000000001</v>
-      </c>
-      <c r="BJ16">
-        <v>-1.17</v>
       </c>
       <c r="BK16">
         <v>-1.17</v>
       </c>
       <c r="BL16">
+        <v>-1.17</v>
+      </c>
+      <c r="BM16">
         <v>-1.01</v>
-      </c>
-      <c r="BM16">
-        <v>-1</v>
       </c>
       <c r="BN16">
         <v>-1</v>
       </c>
       <c r="BO16">
+        <v>-1</v>
+      </c>
+      <c r="BP16">
         <v>-1.01</v>
       </c>
-      <c r="BP16">
+      <c r="BQ16">
         <v>-0.87</v>
       </c>
-      <c r="BQ16">
+      <c r="BR16">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="BR16">
+      <c r="BS16">
         <v>-0.67</v>
       </c>
-      <c r="BS16">
+      <c r="BT16">
         <v>-0.31</v>
       </c>
-      <c r="BT16">
+      <c r="BU16">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="BU16">
+      <c r="BV16">
         <v>-0.5</v>
       </c>
-      <c r="BV16">
+      <c r="BW16">
         <v>-0.36</v>
       </c>
-      <c r="BW16">
+      <c r="BX16">
         <v>-0.48</v>
       </c>
-      <c r="BX16">
+      <c r="BY16">
         <v>-1.35</v>
       </c>
-      <c r="BY16">
+      <c r="BZ16">
         <v>-0.99</v>
       </c>
     </row>
-    <row r="17" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
       <c r="B17">
+        <v>22</v>
+      </c>
+      <c r="C17">
         <v>24</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>28</v>
-      </c>
-      <c r="D17" s="2">
-        <v>22</v>
       </c>
       <c r="E17" s="2">
         <v>22</v>
@@ -4947,16 +4997,16 @@
         <v>22</v>
       </c>
       <c r="G17" s="2">
+        <v>22</v>
+      </c>
+      <c r="H17" s="2">
         <v>24</v>
       </c>
-      <c r="H17" s="2">
+      <c r="I17" s="2">
         <v>21</v>
       </c>
-      <c r="I17" s="2">
+      <c r="J17" s="2">
         <v>14</v>
-      </c>
-      <c r="J17" s="2">
-        <v>20</v>
       </c>
       <c r="K17" s="2">
         <v>20</v>
@@ -4971,10 +5021,10 @@
         <v>20</v>
       </c>
       <c r="O17" s="2">
+        <v>20</v>
+      </c>
+      <c r="P17" s="2">
         <v>15</v>
-      </c>
-      <c r="P17" s="2">
-        <v>20</v>
       </c>
       <c r="Q17" s="2">
         <v>20</v>
@@ -4983,7 +5033,7 @@
         <v>20</v>
       </c>
       <c r="S17" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="T17" s="2">
         <v>18</v>
@@ -4992,13 +5042,13 @@
         <v>18</v>
       </c>
       <c r="V17" s="2">
+        <v>18</v>
+      </c>
+      <c r="W17" s="2">
         <v>13</v>
       </c>
-      <c r="W17" s="2">
+      <c r="X17" s="2">
         <v>14</v>
-      </c>
-      <c r="X17" s="2">
-        <v>22</v>
       </c>
       <c r="Y17" s="2">
         <v>22</v>
@@ -5010,10 +5060,10 @@
         <v>22</v>
       </c>
       <c r="AB17" s="2">
+        <v>22</v>
+      </c>
+      <c r="AC17" s="2">
         <v>21</v>
-      </c>
-      <c r="AC17" s="2">
-        <v>24</v>
       </c>
       <c r="AD17" s="2">
         <v>24</v>
@@ -5025,34 +5075,34 @@
         <v>24</v>
       </c>
       <c r="AG17" s="2">
+        <v>24</v>
+      </c>
+      <c r="AH17" s="2">
         <v>23</v>
       </c>
-      <c r="AH17" s="2">
+      <c r="AI17" s="2">
         <v>22</v>
       </c>
-      <c r="AI17" s="2">
+      <c r="AJ17" s="2">
         <v>28</v>
-      </c>
-      <c r="AJ17" s="2">
-        <v>23</v>
       </c>
       <c r="AK17" s="2">
         <v>23</v>
       </c>
       <c r="AL17" s="2">
+        <v>23</v>
+      </c>
+      <c r="AM17" s="2">
         <v>21</v>
       </c>
-      <c r="AM17" s="2">
+      <c r="AN17" s="2">
         <v>18</v>
       </c>
-      <c r="AN17" s="2">
+      <c r="AO17" s="2">
         <v>17</v>
       </c>
-      <c r="AO17" s="2">
+      <c r="AP17" s="2">
         <v>15</v>
-      </c>
-      <c r="AP17" s="2">
-        <v>22</v>
       </c>
       <c r="AQ17" s="2">
         <v>22</v>
@@ -5064,13 +5114,13 @@
         <v>22</v>
       </c>
       <c r="AT17" s="2">
+        <v>22</v>
+      </c>
+      <c r="AU17" s="2">
         <v>23</v>
       </c>
-      <c r="AU17" s="2">
+      <c r="AV17" s="2">
         <v>19</v>
-      </c>
-      <c r="AV17" s="2">
-        <v>15</v>
       </c>
       <c r="AW17" s="2">
         <v>15</v>
@@ -5079,49 +5129,49 @@
         <v>15</v>
       </c>
       <c r="AY17" s="2">
+        <v>15</v>
+      </c>
+      <c r="AZ17" s="2">
         <v>16</v>
-      </c>
-      <c r="AZ17" s="2">
-        <v>28</v>
       </c>
       <c r="BA17" s="2">
         <v>28</v>
       </c>
       <c r="BB17" s="2">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="BC17" s="2">
         <v>21</v>
       </c>
       <c r="BD17" s="2">
+        <v>21</v>
+      </c>
+      <c r="BE17" s="2">
         <v>22</v>
       </c>
-      <c r="BE17" s="2">
+      <c r="BF17" s="2">
         <v>23</v>
       </c>
-      <c r="BF17" s="2">
+      <c r="BG17" s="2">
         <v>26</v>
       </c>
-      <c r="BG17" s="2">
+      <c r="BH17" s="2">
         <v>28</v>
       </c>
-      <c r="BH17" s="2">
+      <c r="BI17" s="2">
         <v>32</v>
-      </c>
-      <c r="BI17" s="2">
-        <v>34</v>
       </c>
       <c r="BJ17" s="2">
         <v>34</v>
       </c>
       <c r="BK17" s="2">
+        <v>34</v>
+      </c>
+      <c r="BL17" s="2">
         <v>33</v>
       </c>
-      <c r="BL17" s="2">
+      <c r="BM17" s="2">
         <v>22</v>
-      </c>
-      <c r="BM17" s="2">
-        <v>21</v>
       </c>
       <c r="BN17" s="2">
         <v>21</v>
@@ -5130,22 +5180,22 @@
         <v>21</v>
       </c>
       <c r="BP17" s="2">
+        <v>21</v>
+      </c>
+      <c r="BQ17" s="2">
         <v>20</v>
       </c>
-      <c r="BQ17" s="2">
+      <c r="BR17" s="2">
         <v>19</v>
       </c>
-      <c r="BR17" s="2">
+      <c r="BS17" s="2">
         <v>15</v>
       </c>
-      <c r="BS17" s="2">
+      <c r="BT17" s="2">
         <v>19</v>
       </c>
-      <c r="BT17" s="2">
+      <c r="BU17" s="2">
         <v>18</v>
-      </c>
-      <c r="BU17" s="2">
-        <v>16</v>
       </c>
       <c r="BV17" s="2">
         <v>16</v>
@@ -5154,97 +5204,100 @@
         <v>16</v>
       </c>
       <c r="BX17" s="2">
+        <v>16</v>
+      </c>
+      <c r="BY17" s="2">
         <v>15</v>
       </c>
-      <c r="BY17" s="2">
+      <c r="BZ17" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:77" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:78" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
       <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18">
         <v>4</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <v>6</v>
       </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
       <c r="E18" s="2">
         <v>0</v>
       </c>
       <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
         <v>1</v>
       </c>
-      <c r="G18" s="2">
+      <c r="H18" s="2">
         <v>3</v>
       </c>
-      <c r="H18" s="2">
+      <c r="I18" s="2">
         <v>9</v>
       </c>
-      <c r="I18" s="2">
+      <c r="J18" s="2">
         <v>2</v>
       </c>
-      <c r="J18" s="2">
-        <v>0</v>
-      </c>
       <c r="K18" s="2">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2">
         <v>3</v>
       </c>
-      <c r="L18" s="2">
-        <v>0</v>
-      </c>
       <c r="M18" s="2">
+        <v>0</v>
+      </c>
+      <c r="N18" s="2">
         <v>2</v>
       </c>
-      <c r="N18" s="2">
+      <c r="O18" s="2">
         <v>8</v>
       </c>
-      <c r="O18" s="2">
-        <v>0</v>
-      </c>
       <c r="P18" s="2">
         <v>0</v>
       </c>
       <c r="Q18" s="2">
+        <v>0</v>
+      </c>
+      <c r="R18" s="2">
         <v>2</v>
       </c>
-      <c r="R18" s="2">
+      <c r="S18" s="2">
         <v>3</v>
       </c>
-      <c r="S18" s="2">
-        <v>0</v>
-      </c>
       <c r="T18" s="2">
+        <v>0</v>
+      </c>
+      <c r="U18" s="2">
         <v>1</v>
       </c>
-      <c r="U18" s="2">
+      <c r="V18" s="2">
         <v>6</v>
       </c>
-      <c r="V18" s="2">
+      <c r="W18" s="2">
         <v>1</v>
       </c>
-      <c r="W18" s="2">
+      <c r="X18" s="2">
         <v>2</v>
       </c>
-      <c r="X18" s="2">
-        <v>0</v>
-      </c>
       <c r="Y18" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="2">
         <v>2</v>
       </c>
-      <c r="Z18" s="2">
+      <c r="AA18" s="2">
         <v>3</v>
       </c>
-      <c r="AA18" s="2">
+      <c r="AB18" s="2">
         <v>6</v>
       </c>
-      <c r="AB18" s="2">
-        <v>0</v>
-      </c>
       <c r="AC18" s="2">
         <v>0</v>
       </c>
@@ -5252,10 +5305,10 @@
         <v>0</v>
       </c>
       <c r="AE18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="2">
         <v>1</v>
-      </c>
-      <c r="AF18" s="2">
-        <v>2</v>
       </c>
       <c r="AG18" s="2">
         <v>2</v>
@@ -5264,94 +5317,94 @@
         <v>2</v>
       </c>
       <c r="AI18" s="2">
+        <v>2</v>
+      </c>
+      <c r="AJ18" s="2">
         <v>11</v>
       </c>
-      <c r="AJ18" s="2">
+      <c r="AK18" s="2">
         <v>1</v>
       </c>
-      <c r="AK18" s="2">
+      <c r="AL18" s="2">
         <v>2</v>
       </c>
-      <c r="AL18" s="2">
+      <c r="AM18" s="2">
         <v>7</v>
       </c>
-      <c r="AM18" s="2">
+      <c r="AN18" s="2">
         <v>5</v>
       </c>
-      <c r="AN18" s="2">
+      <c r="AO18" s="2">
         <v>4</v>
       </c>
-      <c r="AO18" s="2">
+      <c r="AP18" s="2">
         <v>2</v>
       </c>
-      <c r="AP18" s="2">
+      <c r="AQ18" s="2">
         <v>3</v>
       </c>
-      <c r="AQ18" s="2">
+      <c r="AR18" s="2">
         <v>2</v>
       </c>
-      <c r="AR18" s="2">
+      <c r="AS18" s="2">
         <v>4</v>
       </c>
-      <c r="AS18" s="2">
+      <c r="AT18" s="2">
         <v>2</v>
       </c>
-      <c r="AT18" s="2">
+      <c r="AU18" s="2">
         <v>7</v>
       </c>
-      <c r="AU18" s="2">
+      <c r="AV18" s="2">
         <v>6</v>
       </c>
-      <c r="AV18" s="2">
-        <v>0</v>
-      </c>
       <c r="AW18" s="2">
         <v>0</v>
       </c>
       <c r="AX18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AY18" s="2">
         <v>1</v>
       </c>
-      <c r="AY18" s="2">
+      <c r="AZ18" s="2">
         <v>3</v>
       </c>
-      <c r="AZ18" s="2">
+      <c r="BA18" s="2">
         <v>1</v>
       </c>
-      <c r="BA18" s="2">
+      <c r="BB18" s="2">
         <v>7</v>
       </c>
-      <c r="BB18" s="2">
+      <c r="BC18" s="2">
         <v>2</v>
       </c>
-      <c r="BC18" s="2">
-        <v>0</v>
-      </c>
       <c r="BD18" s="2">
         <v>0</v>
       </c>
       <c r="BE18" s="2">
+        <v>0</v>
+      </c>
+      <c r="BF18" s="2">
         <v>1</v>
       </c>
-      <c r="BF18" s="2">
+      <c r="BG18" s="2">
         <v>3</v>
       </c>
-      <c r="BG18" s="2">
+      <c r="BH18" s="2">
         <v>2</v>
       </c>
-      <c r="BH18" s="2">
+      <c r="BI18" s="2">
         <v>1</v>
       </c>
-      <c r="BI18" s="2">
-        <v>0</v>
-      </c>
       <c r="BJ18" s="2">
+        <v>0</v>
+      </c>
+      <c r="BK18" s="2">
         <v>2</v>
       </c>
-      <c r="BK18" s="2">
+      <c r="BL18" s="2">
         <v>17</v>
-      </c>
-      <c r="BL18" s="2">
-        <v>1</v>
       </c>
       <c r="BM18" s="2">
         <v>1</v>
@@ -5366,34 +5419,37 @@
         <v>1</v>
       </c>
       <c r="BQ18" s="2">
+        <v>1</v>
+      </c>
+      <c r="BR18" s="2">
         <v>4</v>
       </c>
-      <c r="BR18" s="2">
+      <c r="BS18" s="2">
         <v>5</v>
       </c>
-      <c r="BS18" s="2">
+      <c r="BT18" s="2">
         <v>4</v>
       </c>
-      <c r="BT18" s="2">
+      <c r="BU18" s="2">
         <v>2</v>
       </c>
-      <c r="BU18" s="2">
+      <c r="BV18" s="2">
         <v>1</v>
       </c>
-      <c r="BV18" s="2">
-        <v>0</v>
-      </c>
       <c r="BW18" s="2">
+        <v>0</v>
+      </c>
+      <c r="BX18" s="2">
         <v>4</v>
       </c>
-      <c r="BX18" s="2">
+      <c r="BY18" s="2">
         <v>1</v>
       </c>
-      <c r="BY18" s="2">
+      <c r="BZ18" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:77" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:78" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>16</v>
       </c>
@@ -5402,18 +5458,20 @@
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="1:77" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:78" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:F21"/>
+    <mergeCell ref="A20:G21"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>